<commit_message>
API: Implement write data to export excel file
</commit_message>
<xml_diff>
--- a/officedock-api/templates/export/tasks.xlsx
+++ b/officedock-api/templates/export/tasks.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10609"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\マイドライブ\99.OFFICEDOCK\帳票\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/longnguyen/Documents/working/soarig/officedock/source-codes/officedock/officedock-api/templates/export/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1FCE520-545D-4B9D-8844-BC2D11C4143C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8022E070-10E6-8845-B40F-CD83F14913AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{C79B3B14-BDAA-452A-B38D-EDEDE5C344E0}"/>
+    <workbookView xWindow="4020" yWindow="-18840" windowWidth="28800" windowHeight="16040" xr2:uid="{C79B3B14-BDAA-452A-B38D-EDEDE5C344E0}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
   <si>
     <t>サマリー</t>
   </si>
@@ -59,33 +59,18 @@
     <t>期間</t>
   </si>
   <si>
-    <t>2023/04/01 - 2023/04/30</t>
-  </si>
-  <si>
     <t>期間区分</t>
   </si>
   <si>
-    <t>基準期間</t>
-  </si>
-  <si>
     <t>対象ユーザー</t>
   </si>
   <si>
-    <t>田中 太郎</t>
-  </si>
-  <si>
     <t>カテゴリー絞り込み</t>
   </si>
   <si>
-    <t>Aチーム &gt; プロジェクトX &gt; - &gt; -</t>
-  </si>
-  <si>
     <t>タグ絞り込み</t>
   </si>
   <si>
-    <t>#緊急, #要確認</t>
-  </si>
-  <si>
     <t>合計時間</t>
   </si>
   <si>
@@ -99,69 +84,6 @@
   </si>
   <si>
     <t>計測時間</t>
-  </si>
-  <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t>画面仕様書作成</t>
-  </si>
-  <si>
-    <t>40:00:00</t>
-  </si>
-  <si>
-    <t>2</t>
-  </si>
-  <si>
-    <t>API設計レビュー</t>
-  </si>
-  <si>
-    <t>15:30:00</t>
-  </si>
-  <si>
-    <t>3</t>
-  </si>
-  <si>
-    <t>データベース設計</t>
-  </si>
-  <si>
-    <t>35:00:00</t>
-  </si>
-  <si>
-    <t>4</t>
-  </si>
-  <si>
-    <t>チーム週次定例</t>
-  </si>
-  <si>
-    <t>8:00:00</t>
-  </si>
-  <si>
-    <t>5</t>
-  </si>
-  <si>
-    <t>バグ修正作業</t>
-  </si>
-  <si>
-    <t>22:00:00</t>
-  </si>
-  <si>
-    <t>6</t>
-  </si>
-  <si>
-    <t>ドキュメント整理</t>
-  </si>
-  <si>
-    <t>10:00:00</t>
-  </si>
-  <si>
-    <t>7</t>
-  </si>
-  <si>
-    <t>クライアントとの打ち合わせ</t>
-  </si>
-  <si>
-    <t>20:00:00</t>
   </si>
   <si>
     <t>割合</t>
@@ -200,38 +122,7 @@
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>画面設計</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>設計</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>プロジェクトX</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>Aチーム</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>設計レビュー</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>レビュー</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
     <t>タスク集計レポート</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>#緊急 #要確認</t>
-    <rPh sb="5" eb="8">
-      <t>ヨウカクニン</t>
-    </rPh>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -243,14 +134,14 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="游ゴシック"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <charset val="128"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="6"/>
-      <name val="游ゴシック"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <charset val="128"/>
       <scheme val="minor"/>
@@ -259,7 +150,7 @@
       <b/>
       <sz val="16"/>
       <color theme="1"/>
-      <name val="游ゴシック"/>
+      <name val="Calibri"/>
       <family val="3"/>
       <charset val="128"/>
       <scheme val="minor"/>
@@ -268,7 +159,7 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="游ゴシック"/>
+      <name val="Calibri"/>
       <family val="3"/>
       <charset val="128"/>
       <scheme val="minor"/>
@@ -317,7 +208,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -327,27 +218,39 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="46" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="46" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="標準" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -363,9 +266,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office テーマ">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -403,7 +306,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -509,7 +412,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -651,7 +554,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -660,315 +563,179 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C444F05-20AB-4317-94AF-C5FB6B4DC6E3}">
   <dimension ref="A1:I19"/>
-  <sheetFormatPr defaultColWidth="16.19921875" defaultRowHeight="18" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="16.1640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="18.296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.33203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="41" customWidth="1"/>
-    <col min="3" max="4" width="12.5" customWidth="1"/>
+    <col min="3" max="3" width="12.5" customWidth="1"/>
+    <col min="4" max="4" width="12.5" style="9" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="26.4" x14ac:dyDescent="0.45">
-      <c r="A1" s="5" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A2" s="6" t="s">
+    <row r="1" spans="1:9" ht="21" x14ac:dyDescent="0.2">
+      <c r="A1" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1" s="12"/>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A2" s="5" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A3" s="8" t="s">
+      <c r="D2" s="12"/>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A3" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="7" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A4" s="7" t="s">
+      <c r="D3" s="12"/>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A4" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="2"/>
+      <c r="D4" s="12"/>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A5" s="6" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A5" s="7" t="s">
+      <c r="B5" s="2"/>
+      <c r="D5" s="12"/>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A6" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B6" s="2"/>
+      <c r="D6" s="12"/>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A7" s="6" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A6" s="7" t="s">
+      <c r="B7" s="2"/>
+      <c r="D7" s="12"/>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A8" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B8" s="2"/>
+      <c r="D8" s="12"/>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A9" s="6" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A7" s="7" t="s">
+      <c r="B9" s="3"/>
+      <c r="D9" s="12"/>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="D10" s="12"/>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A11" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="D11" s="12"/>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A12" s="7" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A8" s="7" t="s">
+      <c r="B12" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="C12" s="7" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A9" s="7" t="s">
+      <c r="D12" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="B9" s="4">
-        <v>6.270833333333333</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A11" s="6" t="s">
+      <c r="E12" s="7" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A12" s="8" t="s">
+      <c r="F12" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="B12" s="8" t="s">
+      <c r="G12" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="C12" s="8" t="s">
+      <c r="H12" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="D12" s="8" t="s">
-        <v>39</v>
-      </c>
-      <c r="E12" s="8" t="s">
-        <v>40</v>
-      </c>
-      <c r="F12" s="8" t="s">
-        <v>41</v>
-      </c>
-      <c r="G12" s="8" t="s">
-        <v>42</v>
-      </c>
-      <c r="H12" s="8" t="s">
-        <v>43</v>
-      </c>
-      <c r="I12" s="8" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A13" s="1" t="s">
+      <c r="I12" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="B13" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="D13" s="3">
-        <v>0.26600000000000001</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="F13" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="G13" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="H13" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="I13" s="2" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A14" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="D14" s="3">
-        <v>0.10299999999999999</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="F14" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="G14" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="H14" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="I14" s="2" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A15" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="D15" s="3">
-        <v>0.26600000000000001</v>
-      </c>
-      <c r="E15" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="F15" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="G15" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="H15" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="I15" s="2" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A16" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="D16" s="3">
-        <v>0.10299999999999999</v>
-      </c>
-      <c r="E16" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="F16" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="G16" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="H16" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="I16" s="2" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A17" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="D17" s="3">
-        <v>0.26600000000000001</v>
-      </c>
-      <c r="E17" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="F17" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="G17" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="H17" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="I17" s="2" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A18" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="D18" s="3">
-        <v>0.10299999999999999</v>
-      </c>
-      <c r="E18" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="F18" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="G18" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="H18" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="I18" s="2" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A19" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="C19" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="D19" s="3">
-        <v>0.26600000000000001</v>
-      </c>
-      <c r="E19" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="F19" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="G19" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="H19" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="I19" s="2" t="s">
-        <v>52</v>
-      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A13" s="1"/>
+      <c r="B13" s="2"/>
+      <c r="C13" s="2"/>
+      <c r="D13" s="11"/>
+      <c r="E13" s="2"/>
+      <c r="F13" s="2"/>
+      <c r="G13" s="2"/>
+      <c r="H13" s="2"/>
+      <c r="I13" s="2"/>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="B14" s="8"/>
+      <c r="C14" s="8"/>
+      <c r="E14" s="8"/>
+      <c r="F14" s="8"/>
+      <c r="G14" s="8"/>
+      <c r="H14" s="8"/>
+      <c r="I14" s="8"/>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="B15" s="8"/>
+      <c r="C15" s="8"/>
+      <c r="E15" s="8"/>
+      <c r="F15" s="8"/>
+      <c r="G15" s="8"/>
+      <c r="H15" s="8"/>
+      <c r="I15" s="8"/>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="B16" s="8"/>
+      <c r="C16" s="8"/>
+      <c r="E16" s="8"/>
+      <c r="F16" s="8"/>
+      <c r="G16" s="8"/>
+      <c r="H16" s="8"/>
+      <c r="I16" s="8"/>
+    </row>
+    <row r="17" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B17" s="8"/>
+      <c r="C17" s="8"/>
+      <c r="E17" s="8"/>
+      <c r="F17" s="8"/>
+      <c r="G17" s="8"/>
+      <c r="H17" s="8"/>
+      <c r="I17" s="8"/>
+    </row>
+    <row r="18" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B18" s="8"/>
+      <c r="C18" s="8"/>
+      <c r="E18" s="8"/>
+      <c r="F18" s="8"/>
+      <c r="G18" s="8"/>
+      <c r="H18" s="8"/>
+      <c r="I18" s="8"/>
+    </row>
+    <row r="19" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B19" s="8"/>
+      <c r="C19" s="8"/>
+      <c r="E19" s="8"/>
+      <c r="F19" s="8"/>
+      <c r="G19" s="8"/>
+      <c r="H19" s="8"/>
+      <c r="I19" s="8"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1"/>

</xml_diff>

<commit_message>
API: Update export null data of user in statistic
</commit_message>
<xml_diff>
--- a/officedock-api/templates/export/tasks.xlsx
+++ b/officedock-api/templates/export/tasks.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10609"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10308"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/longnguyen/Documents/working/soarig/officedock/source-codes/officedock/officedock-api/templates/export/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/longnguyen/Documents/soarig/projects/officedock/source-codes/officedock/officedock-api/templates/export/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8022E070-10E6-8845-B40F-CD83F14913AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D43AFAB-25E3-E74A-83AB-524BE6208990}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4020" yWindow="-18840" windowWidth="28800" windowHeight="16040" xr2:uid="{C79B3B14-BDAA-452A-B38D-EDEDE5C344E0}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="30240" windowHeight="17340" xr2:uid="{C79B3B14-BDAA-452A-B38D-EDEDE5C344E0}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
   <si>
     <t>サマリー</t>
   </si>
@@ -124,6 +124,9 @@
   <si>
     <t>タスク集計レポート</t>
     <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>対象期間の計測実績がありません</t>
   </si>
 </sst>
 </file>
@@ -208,7 +211,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -244,9 +247,6 @@
     </xf>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -575,13 +575,13 @@
       <c r="A1" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="D1" s="12"/>
+      <c r="D1"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="D2" s="12"/>
+      <c r="D2"/>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3" s="7" t="s">
@@ -590,58 +590,58 @@
       <c r="B3" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="12"/>
+      <c r="D3"/>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" s="6" t="s">
         <v>3</v>
       </c>
       <c r="B4" s="2"/>
-      <c r="D4" s="12"/>
+      <c r="D4"/>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A5" s="6" t="s">
         <v>4</v>
       </c>
       <c r="B5" s="2"/>
-      <c r="D5" s="12"/>
+      <c r="D5"/>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A6" s="6" t="s">
         <v>5</v>
       </c>
       <c r="B6" s="2"/>
-      <c r="D6" s="12"/>
+      <c r="D6"/>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A7" s="6" t="s">
         <v>6</v>
       </c>
       <c r="B7" s="2"/>
-      <c r="D7" s="12"/>
+      <c r="D7"/>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A8" s="6" t="s">
         <v>7</v>
       </c>
       <c r="B8" s="2"/>
-      <c r="D8" s="12"/>
+      <c r="D8"/>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A9" s="6" t="s">
         <v>8</v>
       </c>
       <c r="B9" s="3"/>
-      <c r="D9" s="12"/>
+      <c r="D9"/>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="D10" s="12"/>
+      <c r="D10"/>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A11" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="D11" s="12"/>
+      <c r="D11"/>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A12" s="7" t="s">
@@ -674,7 +674,9 @@
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A13" s="1"/>
-      <c r="B13" s="2"/>
+      <c r="B13" s="2" t="s">
+        <v>20</v>
+      </c>
       <c r="C13" s="2"/>
       <c r="D13" s="11"/>
       <c r="E13" s="2"/>

</xml_diff>